<commit_message>
Vidhan Bhavan Work Name and Subcategory
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="89">
   <si>
     <t>फोटो काढून ४ नग स्टॅम्प साईज फोटो प्रिंटीगसह</t>
   </si>
@@ -27,22 +27,262 @@
     <t>फोटो काढून ४ नग व्‍हीसा साईज फोटो प्रिंटींगसह</t>
   </si>
   <si>
-    <t>फोटोग्राफी ४ तासापर्यंत डाटा डीव्हीडी, सॉफट कॉपी ई-मेलवर अपलोड करणेसह</t>
-  </si>
-  <si>
-    <t>फोटोग्राफी ८ तासापर्यंत डाटा डीव्हीडी, सॉफट कॉपी ई-मेलवर अपलोड करणेसह</t>
-  </si>
-  <si>
-    <t>फोटोग्राफी १२ तासापर्यंत डाटा डीव्हीडी, सॉफट कॉपी ई-मेलवर अपलोड करणेसह</t>
-  </si>
-  <si>
-    <t>मुंबई बाहेर फोटोग्राफी ४ तासापर्यंत डाटा डीव्हीडी, सॉफट कॉपी ई-मेलवर अपलोड करणेसह</t>
-  </si>
-  <si>
-    <t>मुंबई बाहेर फोटोग्राफी ८ तासापर्यंत डाटा डीव्हीडी, सॉफट कॉपी ई-मेलवर अपलोड करणेसह</t>
-  </si>
-  <si>
-    <t>मुंबई बाहेर फोटोग्राफी १२ तासापर्यंत डाटा डीव्हीडी, सॉफट कॉपी ई-मेलवर अपलोड करणेसह</t>
+    <t xml:space="preserve">फोटोग्राफी </t>
+  </si>
+  <si>
+    <t>४ तासापर्यंत डाटा डीव्हीडी, सॉफट कॉपी ई-मेलवर अपलोड करणेसह</t>
+  </si>
+  <si>
+    <t>८ तासापर्यंत डाटा डीव्हीडी, सॉफट कॉपी ई-मेलवर अपलोड करणेसह</t>
+  </si>
+  <si>
+    <t>१२ तासापर्यंत डाटा डीव्हीडी, सॉफट कॉपी ई-मेलवर अपलोड करणेसह</t>
+  </si>
+  <si>
+    <t>मुंबई बाहेर ४ तासापर्यंत डाटा डीव्हीडी, सॉफट कॉपी ई-मेलवर अपलोड करणेसह</t>
+  </si>
+  <si>
+    <t>मुंबई बाहेर ८ तासापर्यंत डाटा डीव्हीडी, सॉफट कॉपी ई-मेलवर अपलोड करणेसह</t>
+  </si>
+  <si>
+    <t>मुंबई बाहेर १२ तासापर्यंत डाटा डीव्हीडी, सॉफट कॉपी ई-मेलवर अपलोड करणेसह</t>
+  </si>
+  <si>
+    <t xml:space="preserve">पासपोर्ट फोटो एक्सपोझिंग चार्जेस सह </t>
+  </si>
+  <si>
+    <t xml:space="preserve">फोटो प्रिंटिंग </t>
+  </si>
+  <si>
+    <t>फोटो अल्बम ( रिकामे )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">२४ X ३० मेट कॉपी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">२० X २४ मेट कॉपी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">१६ X २० मेट कॉपी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">१२ X १८ मेट कॉपी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">१२ X १५ मेट कॉपी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">१० X १२ मेट कॉपी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">८ X १२ मेट कॉपी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">८ X १० मेट कॉपी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">६ X 8 मेट कॉपी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">५ X १० मेट कॉपी अतिरिक्त फोटो </t>
+  </si>
+  <si>
+    <t xml:space="preserve">५ X १० मेट कॉपी </t>
+  </si>
+  <si>
+    <t>५ X ७ साईज अल्बम चार्ज १ X १ ( ४० फोटो )</t>
+  </si>
+  <si>
+    <t>५ X ७ साईज अल्बम चार्ज १ X १ ( ६० फोटो )</t>
+  </si>
+  <si>
+    <t>५ X ७ साईज अल्बम चार्ज १ X १ ( ८० फोटो )</t>
+  </si>
+  <si>
+    <t>५ X ७ साईज अल्बम चार्ज १ X १ ( १०० फोटो )</t>
+  </si>
+  <si>
+    <t>५ X ७ साईज अल्बम चार्ज १ X १ (२०० फोटो )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">१२ X ३६ कव्हर पेज सह कारीजम अल्बम  </t>
+  </si>
+  <si>
+    <t>२५ पाने २०० फोटो  (डिझाईन प्रिंटिंग)</t>
+  </si>
+  <si>
+    <t>१२ X ३६ कारीजम अल्बम १ पाने (डिझाईन प्रिंटिंग)</t>
+  </si>
+  <si>
+    <t>१२ X ३६ कव्हर पेज सह कारीजम अल्बम २५ पाने फक्त प्रिंटिंग)</t>
+  </si>
+  <si>
+    <t>१२ X ३६ कारीजम अल्बम १ पाने फक्त प्रिंटिंग)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">व्हिडिओ शुटींग एक्सपोझिंग चार्जेस सह </t>
+  </si>
+  <si>
+    <t>४ तासपर्यंत (एडिटिंग व डेटा डीव्हीडी सह)</t>
+  </si>
+  <si>
+    <t>८ तासपर्यंत (एडिटिंग व डेटा डीव्हीडी सह)</t>
+  </si>
+  <si>
+    <t>१२ तासपर्यंत (एडिटिंग व डेटा डीव्हीडी सह)</t>
+  </si>
+  <si>
+    <t>मुंबई बाहेर ४ तासपर्यंत (एडिटिंग व डेटा डीव्हीडी सह)</t>
+  </si>
+  <si>
+    <t>मुंबई बाहेर ८ तासपर्यंत (एडिटिंग व डेटा डीव्हीडी सह)</t>
+  </si>
+  <si>
+    <t>मुंबई बाहेर १२ तासपर्यंत (एडिटिंग व डेटा डीव्हीडी सह)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">अतिरिक्त डीव्हीडी कॉपी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">सिंगल डीव्हीडी सेट </t>
+  </si>
+  <si>
+    <t xml:space="preserve">दोन डीव्हीडी सेट </t>
+  </si>
+  <si>
+    <t xml:space="preserve">तीन डीव्हीडी सेट </t>
+  </si>
+  <si>
+    <t xml:space="preserve">चार डीव्हीडी सेट </t>
+  </si>
+  <si>
+    <t xml:space="preserve">पाच डीव्हीडी सेट </t>
+  </si>
+  <si>
+    <t xml:space="preserve">आठ डीव्हीडी सेट </t>
+  </si>
+  <si>
+    <t xml:space="preserve">दहा डीव्हीडी सेट </t>
+  </si>
+  <si>
+    <t xml:space="preserve">१६ जी बी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">३२ जी बी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">६४ जी बी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">१२८ जी बी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">पेनड्राईव ३.० </t>
+  </si>
+  <si>
+    <t xml:space="preserve">हार्डडिस्क </t>
+  </si>
+  <si>
+    <t xml:space="preserve">१ टि. बी. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">२ टि. बी. </t>
+  </si>
+  <si>
+    <t>लाईव्ह व्हिडिओ मिक्सर</t>
+  </si>
+  <si>
+    <t>मुंबई बाहेर लाईव्ह व्हिडिओ मिक्सर</t>
+  </si>
+  <si>
+    <t xml:space="preserve">स्टुडिओ सेटअप चार्जेस </t>
+  </si>
+  <si>
+    <t>स्टुडिओ सेटअप चार्जेस  (दोन लाईट)</t>
+  </si>
+  <si>
+    <t>मुंबई बाहेर स्टुडिओ सेटअप चार्जेस (दोन लाईट)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">सन्माननीय सदस्यांचे एकत्रित छायाचित्र पाकीटासाहित </t>
+  </si>
+  <si>
+    <t xml:space="preserve">सन्माननीय विधानपरिषद सदस्यांचे एकत्रित छायाचित्र (१२ क्ष १५ फोटो साईज व १५ क्ष १८ माउटीग साईज </t>
+  </si>
+  <si>
+    <t xml:space="preserve">सन्माननीय विधानसभा सदस्यांचे एकत्रित छायाचित्र (१८ क्ष २० फोटो साईज व २१ क्ष २४ माउटीग साईज </t>
+  </si>
+  <si>
+    <t xml:space="preserve">सन्माननीय सदस्यांचे एकत्रित छायाचित्र माउटीग सहित (२१  क्ष २४  आकाराचे  माउटीग सहित लाकडी फ्रेम तयार करणे) </t>
+  </si>
+  <si>
+    <t>सनबोर्ड फोटो / लमीनेशन प्रिंटिंगसह ( प्रती चौरस फुट)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">दिवंगत विधानपरिषद व विधानसभा सदस्य यांच्याकरीत स्मृतिपत्र </t>
+  </si>
+  <si>
+    <t>स्मृतिपत्र (गोल्डन एम्बॉस सहित) १२" क्ष १८"</t>
+  </si>
+  <si>
+    <t>आकर्षक फ्रेम माऊंटीग सहित १७" क्ष २३"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">बंद बॉक्स ( १८" क्ष २४" या आकाराचा ) पुरवणे </t>
+  </si>
+  <si>
+    <t xml:space="preserve">फोटो लेमिनेशन </t>
+  </si>
+  <si>
+    <t xml:space="preserve">फोटो सहित लेमिनेशन (लाकडी) प्रती इंच </t>
+  </si>
+  <si>
+    <t xml:space="preserve">फोटो फ्रेम </t>
+  </si>
+  <si>
+    <t>१ इंच लाकडी फ्रेम साईज १०" क्ष १४"</t>
+  </si>
+  <si>
+    <t>१ इंच लाकडी फ्रेम साईज १२" क्ष १४"</t>
+  </si>
+  <si>
+    <t>१ इंच लाकडी फ्रेम साईज १४" क्ष १६"</t>
+  </si>
+  <si>
+    <t>२ इंच लाकडी फ्रेम साईज १४" क्ष २०"</t>
+  </si>
+  <si>
+    <t>२ इंच लाकडी फ्रेम साईज १८" क्ष २२"</t>
+  </si>
+  <si>
+    <t>२.५ इंच लाकडी फ्रेम साईज २२" क्ष २६"</t>
+  </si>
+  <si>
+    <t>२.५ इंच लाकडी फ्रेम साईज २७" क्ष ३३"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">बॅनर </t>
+  </si>
+  <si>
+    <t>डिजिटल फ्लेक्स बॅनर डिझाईन करणे. (प्रती चो. फुट)</t>
+  </si>
+  <si>
+    <t>डिजिटल फ्लेक्स बॅनर डिझाईन प्रिंटिंग सहित (प्रती चो. फुट)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">डिजिटल फ्लेक्स बॅनर डिझाईन प्रिंटिंग/लकडी फ्रेम तयार करणे </t>
+  </si>
+  <si>
+    <t xml:space="preserve">स्टँडीज बॅनर सहित उपलब्घ करून देणे.   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">स्टँडीज लिनेल सहित उपलब्घ करून देणे.  </t>
+  </si>
+  <si>
+    <t>Work Name</t>
+  </si>
+  <si>
+    <t>Work Subcategory</t>
   </si>
 </sst>
 </file>
@@ -81,9 +321,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -378,85 +627,550 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:B11"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="82.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="62.85546875" customWidth="1"/>
+    <col min="3" max="3" width="113.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1">
+    <row r="1" spans="1:3">
+      <c r="B1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="2"/>
+      <c r="C3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="1">
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="1"/>
+      <c r="B4" s="2"/>
+      <c r="C4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="1">
+    </row>
+    <row r="5" spans="1:3">
+      <c r="B5" s="4"/>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="1"/>
+      <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="1">
+      <c r="C6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="1">
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="1"/>
+      <c r="B7" s="2"/>
+      <c r="C7" t="s">
         <v>5</v>
       </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="1">
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="2"/>
+      <c r="C8" t="s">
         <v>6</v>
       </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="1">
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="2"/>
+      <c r="C9" t="s">
         <v>7</v>
       </c>
-      <c r="B9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="1">
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="1"/>
+      <c r="B10" s="2"/>
+      <c r="C10" t="s">
         <v>8</v>
       </c>
-      <c r="B10" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="1">
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="1"/>
+      <c r="B11" s="2"/>
+      <c r="C11" t="s">
         <v>9</v>
       </c>
-      <c r="B11" t="s">
-        <v>8</v>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="1"/>
+      <c r="B12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="1"/>
+      <c r="B13" s="3"/>
+      <c r="C13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="1"/>
+      <c r="B14" s="3"/>
+      <c r="C14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="1"/>
+      <c r="B15" s="3"/>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="1"/>
+      <c r="B16" s="3"/>
+      <c r="C16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="1"/>
+      <c r="B17" s="3"/>
+      <c r="C17" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="1"/>
+      <c r="B18" s="3"/>
+      <c r="C18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="1"/>
+      <c r="B19" s="3"/>
+      <c r="C19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="1"/>
+      <c r="B20" s="3"/>
+      <c r="C20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="1"/>
+      <c r="B21" s="3"/>
+      <c r="C21" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="1"/>
+      <c r="B22" s="3"/>
+      <c r="C22" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="1"/>
+      <c r="B23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="1"/>
+      <c r="B24" s="3"/>
+      <c r="C24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="1"/>
+      <c r="B25" s="3"/>
+      <c r="C25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="1"/>
+      <c r="B26" s="3"/>
+      <c r="C26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="1"/>
+      <c r="B27" s="3"/>
+      <c r="C27" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" s="1"/>
+      <c r="B28" s="3"/>
+      <c r="C28" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="1"/>
+      <c r="B29" s="3"/>
+      <c r="C29" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="1"/>
+      <c r="B30" s="3"/>
+      <c r="C30" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="1"/>
+      <c r="B31" s="3"/>
+      <c r="C31" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" s="1"/>
+      <c r="B32" s="3"/>
+      <c r="C32" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="1"/>
+      <c r="B33" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C33" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="1"/>
+      <c r="B34" s="3"/>
+      <c r="C34" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="1"/>
+      <c r="B35" s="3"/>
+      <c r="C35" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="1"/>
+      <c r="B36" s="3"/>
+      <c r="C36" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" s="1"/>
+      <c r="B37" s="3"/>
+      <c r="C37" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" s="1"/>
+      <c r="B38" s="3"/>
+      <c r="C38" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" s="1"/>
+      <c r="B39" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="B40" s="3"/>
+      <c r="C40" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="B41" s="3"/>
+      <c r="C41" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="B42" s="3"/>
+      <c r="C42" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="B43" s="3"/>
+      <c r="C43" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="B44" s="3"/>
+      <c r="C44" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="B45" s="3"/>
+      <c r="C45" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" s="1"/>
+      <c r="B46" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C46" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="B47" s="3"/>
+      <c r="C47" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="B48" s="3"/>
+      <c r="C48" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="B49" s="3"/>
+      <c r="C49" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" s="1"/>
+      <c r="B50" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C50" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="B51" s="3"/>
+      <c r="C51" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" s="1"/>
+      <c r="B52" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C52" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="B53" s="3"/>
+      <c r="C53" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" s="1"/>
+      <c r="B54" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="B55" s="2"/>
+      <c r="C55" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="B56" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C56" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="B57" s="3"/>
+      <c r="C57" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="B58" s="3"/>
+      <c r="C58" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="B59" s="3"/>
+      <c r="C59" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="B60" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C60" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="B61" s="3"/>
+      <c r="C61" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="B62" s="3"/>
+      <c r="C62" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="B63" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C63" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="B64" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C64" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="65" spans="2:3">
+      <c r="B65" s="3"/>
+      <c r="C65" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="66" spans="2:3">
+      <c r="B66" s="3"/>
+      <c r="C66" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="67" spans="2:3">
+      <c r="B67" s="3"/>
+      <c r="C67" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="68" spans="2:3">
+      <c r="B68" s="3"/>
+      <c r="C68" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="69" spans="2:3">
+      <c r="B69" s="3"/>
+      <c r="C69" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="70" spans="2:3">
+      <c r="B70" s="3"/>
+      <c r="C70" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="71" spans="2:3">
+      <c r="B71" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C71" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="72" spans="2:3">
+      <c r="B72" s="3"/>
+      <c r="C72" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="73" spans="2:3">
+      <c r="B73" s="3"/>
+      <c r="C73" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="74" spans="2:3">
+      <c r="B74" s="3"/>
+      <c r="C74" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="75" spans="2:3">
+      <c r="B75" s="3"/>
+      <c r="C75" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="B33:B38"/>
+    <mergeCell ref="B23:B32"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B6:B11"/>
+    <mergeCell ref="B12:B22"/>
+    <mergeCell ref="B39:B45"/>
+    <mergeCell ref="B71:B75"/>
+    <mergeCell ref="B64:B70"/>
+    <mergeCell ref="B60:B62"/>
+    <mergeCell ref="B56:B59"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="B52:B53"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
added Vidhan Bhavans work name and subcategories
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\Bill Generator Website Final Version\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D610CDC0-00D5-4009-A188-EF34CED9777E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10425" yWindow="90" windowWidth="12465" windowHeight="12345"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -288,11 +294,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-4000439]0"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -309,7 +315,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -317,35 +323,60 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -383,7 +414,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -417,6 +448,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -451,9 +483,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -626,536 +659,543 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C75"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="62.85546875" customWidth="1"/>
-    <col min="3" max="3" width="113.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="62.81640625" customWidth="1"/>
+    <col min="3" max="3" width="113.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="B1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
-      <c r="B3" s="2"/>
-      <c r="C3" t="s">
+      <c r="B3" s="3"/>
+      <c r="C3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
-      <c r="B4" s="2"/>
-      <c r="C4" t="s">
+      <c r="B4" s="3"/>
+      <c r="C4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B5" s="4"/>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="1"/>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>
-      <c r="B7" s="2"/>
-      <c r="C7" t="s">
+      <c r="B7" s="3"/>
+      <c r="C7" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
-      <c r="B8" s="2"/>
-      <c r="C8" t="s">
+      <c r="B8" s="3"/>
+      <c r="C8" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
-      <c r="B9" s="2"/>
-      <c r="C9" t="s">
+      <c r="B9" s="3"/>
+      <c r="C9" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="1"/>
-      <c r="B10" s="2"/>
-      <c r="C10" t="s">
+      <c r="B10" s="3"/>
+      <c r="C10" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
-      <c r="B11" s="2"/>
-      <c r="C11" t="s">
+      <c r="B11" s="3"/>
+      <c r="C11" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
-      <c r="B13" s="3"/>
-      <c r="C13" t="s">
+      <c r="B13" s="5"/>
+      <c r="C13" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
-      <c r="B14" s="3"/>
-      <c r="C14" t="s">
+      <c r="B14" s="5"/>
+      <c r="C14" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
-      <c r="B15" s="3"/>
-      <c r="C15" t="s">
+      <c r="B15" s="5"/>
+      <c r="C15" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
-      <c r="B16" s="3"/>
-      <c r="C16" t="s">
+      <c r="B16" s="5"/>
+      <c r="C16" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
-      <c r="B17" s="3"/>
-      <c r="C17" t="s">
+      <c r="B17" s="5"/>
+      <c r="C17" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
-      <c r="B18" s="3"/>
-      <c r="C18" t="s">
+      <c r="B18" s="5"/>
+      <c r="C18" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
-      <c r="B19" s="3"/>
-      <c r="C19" t="s">
+      <c r="B19" s="5"/>
+      <c r="C19" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
-      <c r="B20" s="3"/>
-      <c r="C20" t="s">
+      <c r="B20" s="5"/>
+      <c r="C20" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
-      <c r="B21" s="3"/>
-      <c r="C21" t="s">
+      <c r="B21" s="5"/>
+      <c r="C21" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
-      <c r="B22" s="3"/>
-      <c r="C22" t="s">
+      <c r="B22" s="5"/>
+      <c r="C22" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="1"/>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
-      <c r="B24" s="3"/>
-      <c r="C24" t="s">
+      <c r="B24" s="5"/>
+      <c r="C24" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
-      <c r="B25" s="3"/>
-      <c r="C25" t="s">
+      <c r="B25" s="5"/>
+      <c r="C25" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
-      <c r="B26" s="3"/>
-      <c r="C26" t="s">
+      <c r="B26" s="5"/>
+      <c r="C26" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
-      <c r="B27" s="3"/>
-      <c r="C27" t="s">
+      <c r="B27" s="5"/>
+      <c r="C27" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
-      <c r="B28" s="3"/>
-      <c r="C28" t="s">
+      <c r="B28" s="5"/>
+      <c r="C28" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
-      <c r="B29" s="3"/>
-      <c r="C29" t="s">
+      <c r="B29" s="5"/>
+      <c r="C29" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
-      <c r="B30" s="3"/>
-      <c r="C30" t="s">
+      <c r="B30" s="5"/>
+      <c r="C30" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="1"/>
-      <c r="B31" s="3"/>
-      <c r="C31" t="s">
+      <c r="B31" s="5"/>
+      <c r="C31" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
-      <c r="B32" s="3"/>
-      <c r="C32" t="s">
+      <c r="B32" s="5"/>
+      <c r="C32" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
-      <c r="B34" s="3"/>
-      <c r="C34" t="s">
+      <c r="B34" s="5"/>
+      <c r="C34" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="1"/>
-      <c r="B35" s="3"/>
-      <c r="C35" t="s">
+      <c r="B35" s="5"/>
+      <c r="C35" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="1"/>
-      <c r="B36" s="3"/>
-      <c r="C36" t="s">
+      <c r="B36" s="5"/>
+      <c r="C36" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="1"/>
-      <c r="B37" s="3"/>
-      <c r="C37" t="s">
+      <c r="B37" s="5"/>
+      <c r="C37" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="1"/>
-      <c r="B38" s="3"/>
-      <c r="C38" t="s">
+      <c r="B38" s="5"/>
+      <c r="C38" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="1"/>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
-      <c r="B40" s="3"/>
-      <c r="C40" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B40" s="5"/>
+      <c r="C40" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
-      <c r="B41" s="3"/>
-      <c r="C41" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B41" s="5"/>
+      <c r="C41" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
-      <c r="B42" s="3"/>
-      <c r="C42" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B42" s="5"/>
+      <c r="C42" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
-      <c r="B43" s="3"/>
-      <c r="C43" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B43" s="5"/>
+      <c r="C43" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
-      <c r="B44" s="3"/>
-      <c r="C44" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B44" s="5"/>
+      <c r="C44" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
-      <c r="B45" s="3"/>
-      <c r="C45" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B45" s="5"/>
+      <c r="C45" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="1"/>
-      <c r="B46" s="3" t="s">
+      <c r="B46" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
-      <c r="B47" s="3"/>
-      <c r="C47" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B47" s="5"/>
+      <c r="C47" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
-      <c r="B48" s="3"/>
-      <c r="C48" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B48" s="5"/>
+      <c r="C48" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
-      <c r="B49" s="3"/>
-      <c r="C49" t="s">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B49" s="5"/>
+      <c r="C49" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="1"/>
-      <c r="B50" s="3" t="s">
+      <c r="B50" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C50" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
-      <c r="B51" s="3"/>
-      <c r="C51" t="s">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B51" s="5"/>
+      <c r="C51" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="1"/>
-      <c r="B52" s="3" t="s">
+      <c r="B52" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C52" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
-      <c r="B53" s="3"/>
-      <c r="C53" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B53" s="5"/>
+      <c r="C53" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="1"/>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C54" s="1" t="s">
+      <c r="C54" s="6" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
-      <c r="B55" s="2"/>
-      <c r="C55" s="1" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B55" s="3"/>
+      <c r="C55" s="6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
-      <c r="B56" s="3" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B56" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C56" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
-      <c r="B57" s="3"/>
-      <c r="C57" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B57" s="5"/>
+      <c r="C57" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="58" spans="1:3">
-      <c r="B58" s="3"/>
-      <c r="C58" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B58" s="5"/>
+      <c r="C58" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
-      <c r="B59" s="3"/>
-      <c r="C59" t="s">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B59" s="5"/>
+      <c r="C59" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
-      <c r="B60" s="3" t="s">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B60" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C60" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="61" spans="1:3">
-      <c r="B61" s="3"/>
-      <c r="C61" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B61" s="5"/>
+      <c r="C61" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="62" spans="1:3">
-      <c r="B62" s="3"/>
-      <c r="C62" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B62" s="5"/>
+      <c r="C62" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="63" spans="1:3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B63" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C63" t="s">
+      <c r="C63" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="64" spans="1:3">
-      <c r="B64" s="3" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B64" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C64" t="s">
+      <c r="C64" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="65" spans="2:3">
-      <c r="B65" s="3"/>
-      <c r="C65" t="s">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B65" s="5"/>
+      <c r="C65" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="66" spans="2:3">
-      <c r="B66" s="3"/>
-      <c r="C66" t="s">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B66" s="5"/>
+      <c r="C66" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="67" spans="2:3">
-      <c r="B67" s="3"/>
-      <c r="C67" t="s">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B67" s="5"/>
+      <c r="C67" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="68" spans="2:3">
-      <c r="B68" s="3"/>
-      <c r="C68" t="s">
+    <row r="68" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B68" s="5"/>
+      <c r="C68" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="69" spans="2:3">
-      <c r="B69" s="3"/>
-      <c r="C69" t="s">
+    <row r="69" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B69" s="5"/>
+      <c r="C69" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="70" spans="2:3">
-      <c r="B70" s="3"/>
-      <c r="C70" t="s">
+    <row r="70" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B70" s="5"/>
+      <c r="C70" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="71" spans="2:3">
-      <c r="B71" s="3" t="s">
+    <row r="71" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B71" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C71" t="s">
+      <c r="C71" s="2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="72" spans="2:3">
-      <c r="B72" s="3"/>
-      <c r="C72" t="s">
+    <row r="72" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B72" s="5"/>
+      <c r="C72" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="73" spans="2:3">
-      <c r="B73" s="3"/>
-      <c r="C73" t="s">
+    <row r="73" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B73" s="5"/>
+      <c r="C73" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="74" spans="2:3">
-      <c r="B74" s="3"/>
-      <c r="C74" t="s">
+    <row r="74" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B74" s="5"/>
+      <c r="C74" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="75" spans="2:3">
-      <c r="B75" s="3"/>
-      <c r="C75" t="s">
+    <row r="75" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B75" s="5"/>
+      <c r="C75" s="2" t="s">
         <v>86</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="B71:B75"/>
+    <mergeCell ref="B64:B70"/>
+    <mergeCell ref="B60:B62"/>
+    <mergeCell ref="B56:B59"/>
+    <mergeCell ref="B54:B55"/>
     <mergeCell ref="B50:B51"/>
     <mergeCell ref="B46:B49"/>
     <mergeCell ref="B33:B38"/>
@@ -1164,30 +1204,24 @@
     <mergeCell ref="B6:B11"/>
     <mergeCell ref="B12:B22"/>
     <mergeCell ref="B39:B45"/>
-    <mergeCell ref="B71:B75"/>
-    <mergeCell ref="B64:B70"/>
-    <mergeCell ref="B60:B62"/>
-    <mergeCell ref="B56:B59"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="B52:B53"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>